<commit_message>
add: Evaluacion de pares
</commit_message>
<xml_diff>
--- a/Evaluacion_de_pares.xlsx
+++ b/Evaluacion_de_pares.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="8">
   <si>
     <t>Entrega 1</t>
   </si>
@@ -41,7 +41,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -64,10 +64,6 @@
       <color rgb="FF000000"/>
       <name val="'Arial'"/>
     </font>
-    <font>
-      <color rgb="FF000000"/>
-      <name val="'Arial'"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -83,7 +79,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -97,7 +93,6 @@
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -393,7 +388,9 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5"/>
+      <c r="A4" s="4" t="s">
+        <v>5</v>
+      </c>
       <c r="B4" s="2"/>
       <c r="C4" s="3">
         <v>20.0</v>

</xml_diff>